<commit_message>
Add diagrams, general PIR-05
</commit_message>
<xml_diff>
--- a/pir_workbook.xlsx
+++ b/pir_workbook.xlsx
@@ -609,12 +609,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Which staff actions (copying files to USB or personal cloud, installing software from untrusted sources) put company data at risk now, and by which routes does it leave?</t>
+          <t>Which new malware families, loaders and attacker techniques are emerging that our detections and hardening should cover?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Which DLP and endpoint controls to prioritise</t>
+          <t>Which detections, hardening steps and log sources to build next</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>insider,insider threat,data exfiltration,data leak,usb,removable media,dlp,shadow it,unauthorized software,trojanized installer,malicious installer,fake installer,cloud storage,data theft</t>
+          <t>new malware,malware family,loader,infostealer,backdoor,remote access trojan,command and control,living off the land,lolbin,powershell,persistence,lateral movement,edr evasion,byovd,sigma rule,yara,detection engineering,mitre att&amp;ck,new technique,campaign,trojanized</t>
         </is>
       </c>
       <c r="H6" t="n">

</xml_diff>

<commit_message>
Drop vulnerability PIR and KEV feed (Stenwatch covers it); four general PIRs; AI summary screenshot
</commit_message>
<xml_diff>
--- a/pir_workbook.xlsx
+++ b/pir_workbook.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -504,17 +504,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Which vulnerabilities in widely deployed edge and enterprise products (VPNs, firewalls, gateways, load balancers, mail and collaboration servers, operating systems) are being exploited now, and which need patching within a day?</t>
+          <t>Which ransomware and extortion groups, and which entry methods, are most active against organisations like ours, and what do they reach first?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Which patches and mitigations to run within a day</t>
+          <t>Which entry-method and recovery controls to prioritise</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>tactical</t>
+          <t>strategic</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -524,7 +524,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>actively exploited,exploited in the wild,known exploited,zero-day,0-day,authentication bypass,remote code execution,vpn,ssl vpn,fortinet,fortigate,fortios,ivanti,palo alto,globalprotect,cisco,citrix,netscaler,f5,big-ip,sonicwall,microsoft exchange,windows,sharepoint,vmware,veeam</t>
+          <t>ransomware,extortion,double extortion,initial access,access broker,data leak site,akira,qilin,lockbit,play,black basta,rhysida,scattered spider,medusa,safepay,emotet,qakbot,dridex,trickbot,icedid,bumblebee,pikabot,lumma</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -539,12 +539,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Which ransomware and extortion groups, and which entry methods, are most active against organisations like ours, and what do they reach first?</t>
+          <t>Which state-aligned and espionage actors are targeting our sector and its supply chain, and through which suppliers or partners do they approach?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Which entry-method and recovery controls to prioritise</t>
+          <t>Supplier and partner risk, customer assurance</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -559,7 +559,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>ransomware,extortion,double extortion,initial access,access broker,data leak site,akira,qilin,lockbit,play,black basta,rhysida,scattered spider,medusa,safepay,emotet,qakbot,dridex,trickbot,icedid,bumblebee,pikabot,lumma</t>
+          <t>state-sponsored,state-aligned,nation-state,espionage,apt28,apt29,apt41,sandworm,turla,lazarus,volt typhoon,salt typhoon,midnight blizzard,russia,china-nexus,north korea,iran,supply chain,critical infrastructure,defence,defense,nato</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -574,17 +574,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Which state-aligned and espionage actors are targeting our sector and its supply chain, and through which suppliers or partners do they approach?</t>
+          <t>Which new malware families, loaders and attacker techniques are emerging that our detections and hardening should cover?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Supplier and partner risk, customer assurance</t>
+          <t>Which detections, hardening steps and log sources to build next</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>strategic</t>
+          <t>tactical</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -594,45 +594,10 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>state-sponsored,state-aligned,nation-state,espionage,apt28,apt29,apt41,sandworm,turla,lazarus,volt typhoon,salt typhoon,midnight blizzard,russia,china-nexus,north korea,iran,supply chain,critical infrastructure,defence,defense,nato</t>
+          <t>new malware,malware family,loader,infostealer,backdoor,remote access trojan,command and control,living off the land,lolbin,powershell,persistence,lateral movement,edr evasion,byovd,sigma rule,yara,detection engineering,mitre att&amp;ck,new technique,campaign,trojanized</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>PIR-05</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Which new malware families, loaders and attacker techniques are emerging that our detections and hardening should cover?</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Which detections, hardening steps and log sources to build next</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>tactical</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Security lead</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>new malware,malware family,loader,infostealer,backdoor,remote access trojan,command and control,living off the land,lolbin,powershell,persistence,lateral movement,edr evasion,byovd,sigma rule,yara,detection engineering,mitre att&amp;ck,new technique,campaign,trojanized</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -647,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -680,71 +645,71 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CISA-KEV</t>
+          <t>DARKREADING</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CISA Known Exploited Vulnerabilities</t>
+          <t>Dark Reading</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>government</t>
+          <t>community</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PIR-02,PIR-03</t>
+          <t>PIR-01,PIR-02,PIR-03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DARKREADING</t>
+          <t>CERT-EU</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dark Reading</t>
+          <t>CERT-EU security advisories</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>community</t>
+          <t>government</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PIR-01,PIR-02,PIR-03,PIR-04</t>
+          <t>PIR-01,PIR-02,PIR-03</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CERT-EU</t>
+          <t>MS-SEC-BLOG</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CERT-EU security advisories</t>
+          <t>Microsoft Security Blog</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>government</t>
+          <t>vendor</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -761,17 +726,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MS-SEC-BLOG</t>
+          <t>DFIR-REPORT</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Microsoft Security Blog</t>
+          <t>The DFIR Report</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>vendor</t>
+          <t>community</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -781,46 +746,46 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PIR-01,PIR-02,PIR-03,PIR-04,PIR-05</t>
+          <t>PIR-01,PIR-02,PIR-04</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DFIR-REPORT</t>
+          <t>CROWDSTRIKE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>The DFIR Report</t>
+          <t>CrowdStrike blog</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>community</t>
+          <t>vendor</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>PIR-01,PIR-03,PIR-05</t>
+          <t>PIR-01,PIR-02,PIR-03</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CROWDSTRIKE</t>
+          <t>UNIT42</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CrowdStrike blog</t>
+          <t>Palo Alto Unit 42</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -835,24 +800,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PIR-01,PIR-03,PIR-04</t>
+          <t>PIR-01,PIR-02,PIR-03,PIR-04</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>UNIT42</t>
+          <t>THN</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Palo Alto Unit 42</t>
+          <t>The Hacker News</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>vendor</t>
+          <t>community</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -862,19 +827,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>PIR-01,PIR-02,PIR-03,PIR-04,PIR-05</t>
+          <t>PIR-01,PIR-02,PIR-03,PIR-04</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>THN</t>
+          <t>FEODO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>The Hacker News</t>
+          <t>abuse.ch Feodo Tracker</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -889,34 +854,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>PIR-01,PIR-02,PIR-03,PIR-04,PIR-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>FEODO</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>abuse.ch Feodo Tracker</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>community</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>PIR-03</t>
+          <t>PIR-02</t>
         </is>
       </c>
     </row>

</xml_diff>